<commit_message>
fix(src): :bug: Update related analysis under the guidance of SYL (2025-05-27, part1)
</commit_message>
<xml_diff>
--- a/output/Tables/mmc1.xlsx
+++ b/output/Tables/mmc1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\luzh29\Library\Projects\WGS_GWAS_and_MR\output\Tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73CA66F7-520E-44BA-9BB8-0EFFD13D540A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88D8432C-2C63-4990-86F5-5E2B9B7EE633}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="692" activeTab="1" xr2:uid="{B1B36BAE-942B-7148-AF58-4A36D0B24BEE}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="16440" windowHeight="28320" tabRatio="692" activeTab="1" xr2:uid="{B1B36BAE-942B-7148-AF58-4A36D0B24BEE}"/>
   </bookViews>
   <sheets>
     <sheet name="Table S1" sheetId="49" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1143" uniqueCount="490">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1154" uniqueCount="501">
   <si>
     <t>Disease</t>
   </si>
@@ -1680,6 +1680,50 @@
   </si>
   <si>
     <t>Descriptions</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Interpolated Year when cancer first diagnosed | Instance 0-3; Coding Meaning: https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=20006</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Interpolated Age of participant when cancer first diagnosed | Instance 0-3; Coding Meaning: https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=20007</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Interpolated Year when non-cancer illness first diagnosed | Instance 0-3; Coding Meaning: https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=20008</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Interpolated Age of participant when non-cancer illness first diagnosed | Instance 0-3; Coding Meaning: https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=20009</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Method of recording time when cancer first diagnosed | Instance 0-3; Coding Meaning: https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=20012</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Method of recording time when non-cancer illness first diagnosed | Instance 0-3; Coding Meaning: https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=20013</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Age at death | Instance 0-1; Coding Meaning: https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=40007</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Age at cancer diagnosis | Instance 0-21; Coding Meaning: https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=40008</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Cancer year/age first occurred | Instance 0-3; Coding Meaning: https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=84</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Non-cancer illness year/age first occurred | Instance 0-3; Coding Meaning: https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=87</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Cancer diagnosed by doctor | Instance 0-3; Coding Meaning: https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=2453</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1896,12 +1940,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1919,6 +1957,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1938,7 +1979,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2324,19 +2368,19 @@
       <c r="C5" s="20">
         <v>1800</v>
       </c>
-      <c r="D5" s="35">
+      <c r="D5" s="34">
         <v>1255</v>
       </c>
-      <c r="E5" s="35" t="s">
+      <c r="E5" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="F5" s="35" t="s">
+      <c r="F5" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="G5" s="35" t="s">
+      <c r="G5" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="H5" s="35">
+      <c r="H5" s="34">
         <v>203972</v>
       </c>
     </row>
@@ -2350,11 +2394,11 @@
       <c r="C6" s="20">
         <v>1801</v>
       </c>
-      <c r="D6" s="35"/>
-      <c r="E6" s="35"/>
-      <c r="F6" s="35"/>
-      <c r="G6" s="35"/>
-      <c r="H6" s="35"/>
+      <c r="D6" s="34"/>
+      <c r="E6" s="34"/>
+      <c r="F6" s="34"/>
+      <c r="G6" s="34"/>
+      <c r="H6" s="34"/>
     </row>
     <row r="7" spans="1:8" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
@@ -2366,11 +2410,11 @@
       <c r="C7" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="35"/>
-      <c r="E7" s="35"/>
-      <c r="F7" s="35"/>
-      <c r="G7" s="35"/>
-      <c r="H7" s="35"/>
+      <c r="D7" s="34"/>
+      <c r="E7" s="34"/>
+      <c r="F7" s="34"/>
+      <c r="G7" s="34"/>
+      <c r="H7" s="34"/>
     </row>
     <row r="8" spans="1:8" s="18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
@@ -2385,10 +2429,10 @@
       <c r="D8" s="3">
         <v>6247</v>
       </c>
-      <c r="E8" s="35"/>
-      <c r="F8" s="35"/>
-      <c r="G8" s="35"/>
-      <c r="H8" s="35"/>
+      <c r="E8" s="34"/>
+      <c r="F8" s="34"/>
+      <c r="G8" s="34"/>
+      <c r="H8" s="34"/>
     </row>
     <row r="9" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
@@ -2400,7 +2444,7 @@
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
-      <c r="H9" s="35"/>
+      <c r="H9" s="34"/>
     </row>
     <row r="10" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
@@ -2415,16 +2459,16 @@
       <c r="D10" s="3">
         <v>2063</v>
       </c>
-      <c r="E10" s="35">
+      <c r="E10" s="34">
         <v>5716</v>
       </c>
-      <c r="F10" s="35" t="s">
+      <c r="F10" s="34" t="s">
         <v>28</v>
       </c>
-      <c r="G10" s="35" t="s">
+      <c r="G10" s="34" t="s">
         <v>27</v>
       </c>
-      <c r="H10" s="35"/>
+      <c r="H10" s="34"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
@@ -2439,10 +2483,10 @@
       <c r="D11" s="3">
         <v>1530</v>
       </c>
-      <c r="E11" s="35"/>
-      <c r="F11" s="35"/>
-      <c r="G11" s="35"/>
-      <c r="H11" s="35"/>
+      <c r="E11" s="34"/>
+      <c r="F11" s="34"/>
+      <c r="G11" s="34"/>
+      <c r="H11" s="34"/>
     </row>
     <row r="12" spans="1:8" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="23" t="s">
@@ -2457,10 +2501,10 @@
       <c r="D12" s="4">
         <v>2269</v>
       </c>
-      <c r="E12" s="36"/>
-      <c r="F12" s="36"/>
-      <c r="G12" s="36"/>
-      <c r="H12" s="36"/>
+      <c r="E12" s="35"/>
+      <c r="F12" s="35"/>
+      <c r="G12" s="35"/>
+      <c r="H12" s="35"/>
     </row>
     <row r="13" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" s="9"/>
@@ -2522,7 +2566,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E85E0DD2-F97D-4D73-B494-1E0809FA7723}">
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.75" style="10" customWidth="1"/>
@@ -2686,120 +2730,208 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="10">
-        <v>40006</v>
+        <v>20006</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>476</v>
+        <v>490</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="10">
-        <v>40013</v>
+        <v>20007</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>477</v>
+        <v>491</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="10">
-        <v>20001</v>
+        <v>20008</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>478</v>
+        <v>492</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="10">
-        <v>40001</v>
+        <v>20009</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>479</v>
+        <v>493</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="10">
-        <v>40002</v>
+        <v>20012</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>480</v>
+        <v>494</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="10">
-        <v>41202</v>
+        <v>20013</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>481</v>
+        <v>495</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="10">
-        <v>41203</v>
+        <v>40007</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>482</v>
+        <v>496</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="10">
-        <v>41204</v>
+        <v>40008</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>483</v>
+        <v>497</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="10">
-        <v>41205</v>
+        <v>84</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>484</v>
+        <v>498</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="10">
-        <v>20002</v>
+        <v>87</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>485</v>
+        <v>499</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="10">
-        <v>41270</v>
+        <v>2453</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>486</v>
+        <v>500</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="10">
+        <v>40006</v>
+      </c>
+      <c r="B31" s="12" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" s="10">
+        <v>40013</v>
+      </c>
+      <c r="B32" s="12" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" s="10">
+        <v>20001</v>
+      </c>
+      <c r="B33" s="12" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" s="10">
+        <v>40001</v>
+      </c>
+      <c r="B34" s="12" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" s="10">
+        <v>40002</v>
+      </c>
+      <c r="B35" s="12" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" s="10">
+        <v>41202</v>
+      </c>
+      <c r="B36" s="12" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" s="10">
+        <v>41203</v>
+      </c>
+      <c r="B37" s="12" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" s="10">
+        <v>41204</v>
+      </c>
+      <c r="B38" s="12" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" s="10">
+        <v>41205</v>
+      </c>
+      <c r="B39" s="12" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" s="10">
+        <v>20002</v>
+      </c>
+      <c r="B40" s="12" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" s="10">
+        <v>41270</v>
+      </c>
+      <c r="B41" s="12" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" s="10">
         <v>41271</v>
       </c>
-      <c r="B31" s="12" t="s">
+      <c r="B42" s="12" t="s">
         <v>487</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="41">
+    <row r="43" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="33">
         <v>1647</v>
       </c>
-      <c r="B32" s="32" t="s">
+      <c r="B43" s="30" t="s">
         <v>488</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A34" s="10" t="s">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" s="10" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A35" s="10" t="s">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" s="10" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A36" s="12" t="s">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" s="12" t="s">
         <v>33</v>
       </c>
     </row>
@@ -2832,7 +2964,7 @@
         <v>455</v>
       </c>
       <c r="C1" s="2"/>
-      <c r="D1" s="30"/>
+      <c r="D1" s="28"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
@@ -2841,25 +2973,25 @@
     </row>
     <row r="2" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:9" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="27" t="s">
+      <c r="A3" s="40" t="s">
         <v>128</v>
       </c>
-      <c r="B3" s="27" t="s">
+      <c r="B3" s="40" t="s">
         <v>304</v>
       </c>
-      <c r="C3" s="37" t="s">
+      <c r="C3" s="36" t="s">
         <v>155</v>
       </c>
-      <c r="D3" s="37"/>
-      <c r="E3" s="37"/>
-      <c r="F3" s="37"/>
+      <c r="D3" s="36"/>
+      <c r="E3" s="36"/>
+      <c r="F3" s="36"/>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
     </row>
     <row r="4" spans="1:9" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="28"/>
-      <c r="B4" s="28"/>
+      <c r="A4" s="41"/>
+      <c r="B4" s="41"/>
       <c r="C4" s="6" t="s">
         <v>129</v>
       </c>
@@ -2877,7 +3009,7 @@
       <c r="I4" s="2"/>
     </row>
     <row r="5" spans="1:9" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="38" t="s">
+      <c r="A5" s="37" t="s">
         <v>157</v>
       </c>
       <c r="B5" s="9" t="s">
@@ -2886,7 +3018,7 @@
       <c r="C5" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="D5" s="29" t="s">
+      <c r="D5" s="27" t="s">
         <v>164</v>
       </c>
       <c r="E5" s="2"/>
@@ -2898,7 +3030,7 @@
       <c r="I5" s="2"/>
     </row>
     <row r="6" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="39"/>
+      <c r="A6" s="38"/>
       <c r="B6" s="12" t="s">
         <v>167</v>
       </c>
@@ -2916,7 +3048,7 @@
       </c>
     </row>
     <row r="7" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="39"/>
+      <c r="A7" s="38"/>
       <c r="B7" s="12" t="s">
         <v>131</v>
       </c>
@@ -2934,7 +3066,7 @@
       </c>
     </row>
     <row r="8" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="39"/>
+      <c r="A8" s="38"/>
       <c r="B8" s="12" t="s">
         <v>168</v>
       </c>
@@ -2952,7 +3084,7 @@
       </c>
     </row>
     <row r="9" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="39"/>
+      <c r="A9" s="38"/>
       <c r="B9" s="12" t="s">
         <v>131</v>
       </c>
@@ -2970,7 +3102,7 @@
       </c>
     </row>
     <row r="10" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="39"/>
+      <c r="A10" s="38"/>
       <c r="B10" s="12" t="s">
         <v>297</v>
       </c>
@@ -2988,7 +3120,7 @@
       </c>
     </row>
     <row r="11" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="39"/>
+      <c r="A11" s="38"/>
       <c r="B11" s="12" t="s">
         <v>131</v>
       </c>
@@ -3006,7 +3138,7 @@
       </c>
     </row>
     <row r="12" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="39"/>
+      <c r="A12" s="38"/>
       <c r="B12" s="12" t="s">
         <v>158</v>
       </c>
@@ -3024,7 +3156,7 @@
       </c>
     </row>
     <row r="13" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="39"/>
+      <c r="A13" s="38"/>
       <c r="B13" s="12" t="s">
         <v>132</v>
       </c>
@@ -3042,7 +3174,7 @@
       </c>
     </row>
     <row r="14" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="39"/>
+      <c r="A14" s="38"/>
       <c r="B14" s="12" t="s">
         <v>133</v>
       </c>
@@ -3060,7 +3192,7 @@
       </c>
     </row>
     <row r="15" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="39"/>
+      <c r="A15" s="38"/>
       <c r="B15" s="12" t="s">
         <v>134</v>
       </c>
@@ -3078,7 +3210,7 @@
       </c>
     </row>
     <row r="16" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="39"/>
+      <c r="A16" s="38"/>
       <c r="B16" s="12" t="s">
         <v>135</v>
       </c>
@@ -3096,7 +3228,7 @@
       </c>
     </row>
     <row r="17" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="39"/>
+      <c r="A17" s="38"/>
       <c r="B17" s="12" t="s">
         <v>136</v>
       </c>
@@ -3114,7 +3246,7 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="39"/>
+      <c r="A18" s="38"/>
       <c r="B18" s="12" t="s">
         <v>137</v>
       </c>
@@ -3132,7 +3264,7 @@
       </c>
     </row>
     <row r="19" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="39"/>
+      <c r="A19" s="38"/>
       <c r="B19" s="12" t="s">
         <v>138</v>
       </c>
@@ -3150,7 +3282,7 @@
       </c>
     </row>
     <row r="20" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="39"/>
+      <c r="A20" s="38"/>
       <c r="B20" s="12" t="s">
         <v>159</v>
       </c>
@@ -3168,7 +3300,7 @@
       </c>
     </row>
     <row r="21" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="39"/>
+      <c r="A21" s="38"/>
       <c r="B21" s="12" t="s">
         <v>139</v>
       </c>
@@ -3186,7 +3318,7 @@
       </c>
     </row>
     <row r="22" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="39"/>
+      <c r="A22" s="38"/>
       <c r="B22" s="12" t="s">
         <v>140</v>
       </c>
@@ -3204,7 +3336,7 @@
       </c>
     </row>
     <row r="23" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="39"/>
+      <c r="A23" s="38"/>
       <c r="B23" s="12" t="s">
         <v>160</v>
       </c>
@@ -3222,7 +3354,7 @@
       </c>
     </row>
     <row r="24" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="39"/>
+      <c r="A24" s="38"/>
       <c r="B24" s="12" t="s">
         <v>141</v>
       </c>
@@ -3240,7 +3372,7 @@
       </c>
     </row>
     <row r="25" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="39"/>
+      <c r="A25" s="38"/>
       <c r="B25" s="12" t="s">
         <v>142</v>
       </c>
@@ -3258,7 +3390,7 @@
       </c>
     </row>
     <row r="26" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="39"/>
+      <c r="A26" s="38"/>
       <c r="B26" s="12" t="s">
         <v>143</v>
       </c>
@@ -3276,7 +3408,7 @@
       </c>
     </row>
     <row r="27" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="39"/>
+      <c r="A27" s="38"/>
       <c r="B27" s="12" t="s">
         <v>138</v>
       </c>
@@ -3294,7 +3426,7 @@
       </c>
     </row>
     <row r="28" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="39"/>
+      <c r="A28" s="38"/>
       <c r="B28" s="12" t="s">
         <v>161</v>
       </c>
@@ -3312,7 +3444,7 @@
       </c>
     </row>
     <row r="29" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="39"/>
+      <c r="A29" s="38"/>
       <c r="B29" s="12" t="s">
         <v>144</v>
       </c>
@@ -3330,7 +3462,7 @@
       </c>
     </row>
     <row r="30" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="39"/>
+      <c r="A30" s="38"/>
       <c r="B30" s="12" t="s">
         <v>145</v>
       </c>
@@ -3348,7 +3480,7 @@
       </c>
     </row>
     <row r="31" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="39"/>
+      <c r="A31" s="38"/>
       <c r="B31" s="12" t="s">
         <v>146</v>
       </c>
@@ -3366,7 +3498,7 @@
       </c>
     </row>
     <row r="32" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="39"/>
+      <c r="A32" s="38"/>
       <c r="B32" s="12" t="s">
         <v>147</v>
       </c>
@@ -3384,7 +3516,7 @@
       </c>
     </row>
     <row r="33" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="39"/>
+      <c r="A33" s="38"/>
       <c r="B33" s="12" t="s">
         <v>148</v>
       </c>
@@ -3402,7 +3534,7 @@
       </c>
     </row>
     <row r="34" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="39"/>
+      <c r="A34" s="38"/>
       <c r="B34" s="12" t="s">
         <v>141</v>
       </c>
@@ -3420,7 +3552,7 @@
       </c>
     </row>
     <row r="35" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="39"/>
+      <c r="A35" s="38"/>
       <c r="B35" s="12" t="s">
         <v>138</v>
       </c>
@@ -3438,7 +3570,7 @@
       </c>
     </row>
     <row r="36" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="39"/>
+      <c r="A36" s="38"/>
       <c r="B36" s="12" t="s">
         <v>162</v>
       </c>
@@ -3456,7 +3588,7 @@
       </c>
     </row>
     <row r="37" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="39"/>
+      <c r="A37" s="38"/>
       <c r="B37" s="12" t="s">
         <v>149</v>
       </c>
@@ -3474,7 +3606,7 @@
       </c>
     </row>
     <row r="38" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="39"/>
+      <c r="A38" s="38"/>
       <c r="B38" s="12" t="s">
         <v>150</v>
       </c>
@@ -3492,7 +3624,7 @@
       </c>
     </row>
     <row r="39" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="39"/>
+      <c r="A39" s="38"/>
       <c r="B39" s="12" t="s">
         <v>138</v>
       </c>
@@ -3510,7 +3642,7 @@
       </c>
     </row>
     <row r="40" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="39"/>
+      <c r="A40" s="38"/>
       <c r="B40" s="12" t="s">
         <v>163</v>
       </c>
@@ -3528,7 +3660,7 @@
       </c>
     </row>
     <row r="41" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="39"/>
+      <c r="A41" s="38"/>
       <c r="B41" s="12" t="s">
         <v>151</v>
       </c>
@@ -3546,7 +3678,7 @@
       </c>
     </row>
     <row r="42" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="39"/>
+      <c r="A42" s="38"/>
       <c r="B42" s="12" t="s">
         <v>152</v>
       </c>
@@ -3564,7 +3696,7 @@
       </c>
     </row>
     <row r="43" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="39"/>
+      <c r="A43" s="38"/>
       <c r="B43" s="12" t="s">
         <v>153</v>
       </c>
@@ -3582,7 +3714,7 @@
       </c>
     </row>
     <row r="44" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="39"/>
+      <c r="A44" s="38"/>
       <c r="B44" s="12" t="s">
         <v>154</v>
       </c>
@@ -3600,7 +3732,7 @@
       </c>
     </row>
     <row r="45" spans="1:9" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A45" s="39" t="s">
+      <c r="A45" s="38" t="s">
         <v>169</v>
       </c>
       <c r="B45" s="9" t="s">
@@ -3609,7 +3741,7 @@
       <c r="C45" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="D45" s="30" t="s">
+      <c r="D45" s="28" t="s">
         <v>171</v>
       </c>
       <c r="E45" s="2"/>
@@ -3621,7 +3753,7 @@
       <c r="I45" s="2"/>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A46" s="39"/>
+      <c r="A46" s="38"/>
       <c r="B46" s="12" t="s">
         <v>167</v>
       </c>
@@ -3639,7 +3771,7 @@
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A47" s="39"/>
+      <c r="A47" s="38"/>
       <c r="B47" s="12" t="s">
         <v>131</v>
       </c>
@@ -3657,7 +3789,7 @@
       </c>
     </row>
     <row r="48" spans="1:9" ht="18" x14ac:dyDescent="0.25">
-      <c r="A48" s="39"/>
+      <c r="A48" s="38"/>
       <c r="B48" s="12" t="s">
         <v>168</v>
       </c>
@@ -3675,7 +3807,7 @@
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A49" s="39"/>
+      <c r="A49" s="38"/>
       <c r="B49" s="12" t="s">
         <v>131</v>
       </c>
@@ -3693,7 +3825,7 @@
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A50" s="39"/>
+      <c r="A50" s="38"/>
       <c r="B50" s="12" t="s">
         <v>297</v>
       </c>
@@ -3711,7 +3843,7 @@
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A51" s="39"/>
+      <c r="A51" s="38"/>
       <c r="B51" s="12" t="s">
         <v>131</v>
       </c>
@@ -3729,7 +3861,7 @@
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A52" s="39"/>
+      <c r="A52" s="38"/>
       <c r="B52" s="12" t="s">
         <v>158</v>
       </c>
@@ -3747,7 +3879,7 @@
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A53" s="39"/>
+      <c r="A53" s="38"/>
       <c r="B53" s="12" t="s">
         <v>132</v>
       </c>
@@ -3765,7 +3897,7 @@
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A54" s="39"/>
+      <c r="A54" s="38"/>
       <c r="B54" s="12" t="s">
         <v>133</v>
       </c>
@@ -3783,7 +3915,7 @@
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A55" s="39"/>
+      <c r="A55" s="38"/>
       <c r="B55" s="12" t="s">
         <v>134</v>
       </c>
@@ -3801,7 +3933,7 @@
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A56" s="39"/>
+      <c r="A56" s="38"/>
       <c r="B56" s="12" t="s">
         <v>135</v>
       </c>
@@ -3819,7 +3951,7 @@
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A57" s="39"/>
+      <c r="A57" s="38"/>
       <c r="B57" s="12" t="s">
         <v>136</v>
       </c>
@@ -3837,7 +3969,7 @@
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A58" s="39"/>
+      <c r="A58" s="38"/>
       <c r="B58" s="12" t="s">
         <v>137</v>
       </c>
@@ -3855,7 +3987,7 @@
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A59" s="39"/>
+      <c r="A59" s="38"/>
       <c r="B59" s="12" t="s">
         <v>138</v>
       </c>
@@ -3873,7 +4005,7 @@
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A60" s="39"/>
+      <c r="A60" s="38"/>
       <c r="B60" s="12" t="s">
         <v>159</v>
       </c>
@@ -3891,7 +4023,7 @@
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A61" s="39"/>
+      <c r="A61" s="38"/>
       <c r="B61" s="12" t="s">
         <v>139</v>
       </c>
@@ -3909,7 +4041,7 @@
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A62" s="39"/>
+      <c r="A62" s="38"/>
       <c r="B62" s="12" t="s">
         <v>140</v>
       </c>
@@ -3927,7 +4059,7 @@
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A63" s="39"/>
+      <c r="A63" s="38"/>
       <c r="B63" s="12" t="s">
         <v>160</v>
       </c>
@@ -3945,7 +4077,7 @@
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A64" s="39"/>
+      <c r="A64" s="38"/>
       <c r="B64" s="12" t="s">
         <v>141</v>
       </c>
@@ -3963,7 +4095,7 @@
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A65" s="39"/>
+      <c r="A65" s="38"/>
       <c r="B65" s="12" t="s">
         <v>142</v>
       </c>
@@ -3981,7 +4113,7 @@
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A66" s="39"/>
+      <c r="A66" s="38"/>
       <c r="B66" s="12" t="s">
         <v>143</v>
       </c>
@@ -3999,7 +4131,7 @@
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A67" s="39"/>
+      <c r="A67" s="38"/>
       <c r="B67" s="12" t="s">
         <v>138</v>
       </c>
@@ -4017,7 +4149,7 @@
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A68" s="39"/>
+      <c r="A68" s="38"/>
       <c r="B68" s="12" t="s">
         <v>161</v>
       </c>
@@ -4035,7 +4167,7 @@
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A69" s="39"/>
+      <c r="A69" s="38"/>
       <c r="B69" s="12" t="s">
         <v>144</v>
       </c>
@@ -4053,7 +4185,7 @@
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A70" s="39"/>
+      <c r="A70" s="38"/>
       <c r="B70" s="12" t="s">
         <v>145</v>
       </c>
@@ -4071,7 +4203,7 @@
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A71" s="39"/>
+      <c r="A71" s="38"/>
       <c r="B71" s="12" t="s">
         <v>146</v>
       </c>
@@ -4089,7 +4221,7 @@
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A72" s="39"/>
+      <c r="A72" s="38"/>
       <c r="B72" s="12" t="s">
         <v>147</v>
       </c>
@@ -4107,7 +4239,7 @@
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A73" s="39"/>
+      <c r="A73" s="38"/>
       <c r="B73" s="12" t="s">
         <v>148</v>
       </c>
@@ -4125,7 +4257,7 @@
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A74" s="39"/>
+      <c r="A74" s="38"/>
       <c r="B74" s="12" t="s">
         <v>141</v>
       </c>
@@ -4143,7 +4275,7 @@
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A75" s="39"/>
+      <c r="A75" s="38"/>
       <c r="B75" s="12" t="s">
         <v>138</v>
       </c>
@@ -4161,7 +4293,7 @@
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A76" s="39"/>
+      <c r="A76" s="38"/>
       <c r="B76" s="12" t="s">
         <v>162</v>
       </c>
@@ -4179,7 +4311,7 @@
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A77" s="39"/>
+      <c r="A77" s="38"/>
       <c r="B77" s="12" t="s">
         <v>149</v>
       </c>
@@ -4197,7 +4329,7 @@
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A78" s="39"/>
+      <c r="A78" s="38"/>
       <c r="B78" s="12" t="s">
         <v>150</v>
       </c>
@@ -4215,7 +4347,7 @@
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A79" s="39"/>
+      <c r="A79" s="38"/>
       <c r="B79" s="12" t="s">
         <v>138</v>
       </c>
@@ -4233,7 +4365,7 @@
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A80" s="39"/>
+      <c r="A80" s="38"/>
       <c r="B80" s="12" t="s">
         <v>163</v>
       </c>
@@ -4251,7 +4383,7 @@
       </c>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A81" s="39"/>
+      <c r="A81" s="38"/>
       <c r="B81" s="12" t="s">
         <v>151</v>
       </c>
@@ -4269,7 +4401,7 @@
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A82" s="39"/>
+      <c r="A82" s="38"/>
       <c r="B82" s="12" t="s">
         <v>152</v>
       </c>
@@ -4287,7 +4419,7 @@
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A83" s="39"/>
+      <c r="A83" s="38"/>
       <c r="B83" s="12" t="s">
         <v>153</v>
       </c>
@@ -4305,7 +4437,7 @@
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A84" s="39"/>
+      <c r="A84" s="38"/>
       <c r="B84" s="12" t="s">
         <v>154</v>
       </c>
@@ -4323,7 +4455,7 @@
       </c>
     </row>
     <row r="85" spans="1:9" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A85" s="39" t="s">
+      <c r="A85" s="38" t="s">
         <v>236</v>
       </c>
       <c r="B85" s="9" t="s">
@@ -4332,7 +4464,7 @@
       <c r="C85" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="D85" s="29" t="s">
+      <c r="D85" s="27" t="s">
         <v>171</v>
       </c>
       <c r="E85" s="2"/>
@@ -4344,14 +4476,14 @@
       <c r="I85" s="2"/>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A86" s="39"/>
+      <c r="A86" s="38"/>
       <c r="B86" s="12" t="s">
         <v>167</v>
       </c>
       <c r="C86" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D86" s="31" t="s">
+      <c r="D86" s="29" t="s">
         <v>35</v>
       </c>
       <c r="E86" s="1" t="s">
@@ -4362,14 +4494,14 @@
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A87" s="39"/>
+      <c r="A87" s="38"/>
       <c r="B87" s="12" t="s">
         <v>131</v>
       </c>
       <c r="C87" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="D87" s="31" t="s">
+      <c r="D87" s="29" t="s">
         <v>38</v>
       </c>
       <c r="E87" s="1" t="s">
@@ -4380,14 +4512,14 @@
       </c>
     </row>
     <row r="88" spans="1:9" ht="18" x14ac:dyDescent="0.25">
-      <c r="A88" s="39"/>
+      <c r="A88" s="38"/>
       <c r="B88" s="12" t="s">
         <v>168</v>
       </c>
       <c r="C88" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D88" s="31" t="s">
+      <c r="D88" s="29" t="s">
         <v>35</v>
       </c>
       <c r="E88" s="1" t="s">
@@ -4398,14 +4530,14 @@
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A89" s="39"/>
+      <c r="A89" s="38"/>
       <c r="B89" s="12" t="s">
         <v>131</v>
       </c>
       <c r="C89" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="D89" s="31" t="s">
+      <c r="D89" s="29" t="s">
         <v>41</v>
       </c>
       <c r="E89" s="1" t="s">
@@ -4416,14 +4548,14 @@
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A90" s="39"/>
+      <c r="A90" s="38"/>
       <c r="B90" s="12" t="s">
         <v>297</v>
       </c>
       <c r="C90" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D90" s="31" t="s">
+      <c r="D90" s="29" t="s">
         <v>35</v>
       </c>
       <c r="E90" s="1" t="s">
@@ -4434,14 +4566,14 @@
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A91" s="39"/>
+      <c r="A91" s="38"/>
       <c r="B91" s="12" t="s">
         <v>131</v>
       </c>
       <c r="C91" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="D91" s="31" t="s">
+      <c r="D91" s="29" t="s">
         <v>44</v>
       </c>
       <c r="E91" s="1" t="s">
@@ -4452,14 +4584,14 @@
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A92" s="39"/>
+      <c r="A92" s="38"/>
       <c r="B92" s="12" t="s">
         <v>158</v>
       </c>
       <c r="C92" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D92" s="31" t="s">
+      <c r="D92" s="29" t="s">
         <v>35</v>
       </c>
       <c r="E92" s="1" t="s">
@@ -4470,14 +4602,14 @@
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A93" s="39"/>
+      <c r="A93" s="38"/>
       <c r="B93" s="12" t="s">
         <v>132</v>
       </c>
       <c r="C93" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="D93" s="31" t="s">
+      <c r="D93" s="29" t="s">
         <v>47</v>
       </c>
       <c r="E93" s="1" t="s">
@@ -4488,14 +4620,14 @@
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A94" s="39"/>
+      <c r="A94" s="38"/>
       <c r="B94" s="12" t="s">
         <v>133</v>
       </c>
       <c r="C94" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="D94" s="31" t="s">
+      <c r="D94" s="29" t="s">
         <v>50</v>
       </c>
       <c r="E94" s="1" t="s">
@@ -4506,14 +4638,14 @@
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A95" s="39"/>
+      <c r="A95" s="38"/>
       <c r="B95" s="12" t="s">
         <v>134</v>
       </c>
       <c r="C95" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="D95" s="31" t="s">
+      <c r="D95" s="29" t="s">
         <v>53</v>
       </c>
       <c r="E95" s="1" t="s">
@@ -4524,14 +4656,14 @@
       </c>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A96" s="39"/>
+      <c r="A96" s="38"/>
       <c r="B96" s="12" t="s">
         <v>135</v>
       </c>
       <c r="C96" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="D96" s="31" t="s">
+      <c r="D96" s="29" t="s">
         <v>56</v>
       </c>
       <c r="E96" s="1" t="s">
@@ -4542,14 +4674,14 @@
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A97" s="39"/>
+      <c r="A97" s="38"/>
       <c r="B97" s="12" t="s">
         <v>136</v>
       </c>
       <c r="C97" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="D97" s="31" t="s">
+      <c r="D97" s="29" t="s">
         <v>59</v>
       </c>
       <c r="E97" s="1" t="s">
@@ -4560,14 +4692,14 @@
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A98" s="39"/>
+      <c r="A98" s="38"/>
       <c r="B98" s="12" t="s">
         <v>137</v>
       </c>
       <c r="C98" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="D98" s="31" t="s">
+      <c r="D98" s="29" t="s">
         <v>62</v>
       </c>
       <c r="E98" s="1" t="s">
@@ -4578,14 +4710,14 @@
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A99" s="39"/>
+      <c r="A99" s="38"/>
       <c r="B99" s="12" t="s">
         <v>138</v>
       </c>
       <c r="C99" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="D99" s="31" t="s">
+      <c r="D99" s="29" t="s">
         <v>65</v>
       </c>
       <c r="E99" s="1" t="s">
@@ -4596,14 +4728,14 @@
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A100" s="39"/>
+      <c r="A100" s="38"/>
       <c r="B100" s="12" t="s">
         <v>159</v>
       </c>
       <c r="C100" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D100" s="31" t="s">
+      <c r="D100" s="29" t="s">
         <v>35</v>
       </c>
       <c r="E100" s="1" t="s">
@@ -4614,14 +4746,14 @@
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A101" s="39"/>
+      <c r="A101" s="38"/>
       <c r="B101" s="12" t="s">
         <v>139</v>
       </c>
       <c r="C101" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="D101" s="31" t="s">
+      <c r="D101" s="29" t="s">
         <v>68</v>
       </c>
       <c r="E101" s="1" t="s">
@@ -4632,14 +4764,14 @@
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A102" s="39"/>
+      <c r="A102" s="38"/>
       <c r="B102" s="12" t="s">
         <v>140</v>
       </c>
       <c r="C102" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="D102" s="31" t="s">
+      <c r="D102" s="29" t="s">
         <v>71</v>
       </c>
       <c r="E102" s="1" t="s">
@@ -4650,14 +4782,14 @@
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A103" s="39"/>
+      <c r="A103" s="38"/>
       <c r="B103" s="12" t="s">
         <v>160</v>
       </c>
       <c r="C103" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D103" s="31" t="s">
+      <c r="D103" s="29" t="s">
         <v>35</v>
       </c>
       <c r="E103" s="1" t="s">
@@ -4668,14 +4800,14 @@
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A104" s="39"/>
+      <c r="A104" s="38"/>
       <c r="B104" s="12" t="s">
         <v>141</v>
       </c>
       <c r="C104" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="D104" s="31" t="s">
+      <c r="D104" s="29" t="s">
         <v>74</v>
       </c>
       <c r="E104" s="1" t="s">
@@ -4686,14 +4818,14 @@
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A105" s="39"/>
+      <c r="A105" s="38"/>
       <c r="B105" s="12" t="s">
         <v>142</v>
       </c>
       <c r="C105" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="D105" s="31" t="s">
+      <c r="D105" s="29" t="s">
         <v>77</v>
       </c>
       <c r="E105" s="1" t="s">
@@ -4704,14 +4836,14 @@
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A106" s="39"/>
+      <c r="A106" s="38"/>
       <c r="B106" s="12" t="s">
         <v>143</v>
       </c>
       <c r="C106" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="D106" s="31" t="s">
+      <c r="D106" s="29" t="s">
         <v>80</v>
       </c>
       <c r="E106" s="1" t="s">
@@ -4722,14 +4854,14 @@
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A107" s="39"/>
+      <c r="A107" s="38"/>
       <c r="B107" s="12" t="s">
         <v>138</v>
       </c>
       <c r="C107" s="1" t="s">
         <v>267</v>
       </c>
-      <c r="D107" s="31" t="s">
+      <c r="D107" s="29" t="s">
         <v>83</v>
       </c>
       <c r="E107" s="1" t="s">
@@ -4740,14 +4872,14 @@
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A108" s="39"/>
+      <c r="A108" s="38"/>
       <c r="B108" s="12" t="s">
         <v>161</v>
       </c>
       <c r="C108" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D108" s="31" t="s">
+      <c r="D108" s="29" t="s">
         <v>35</v>
       </c>
       <c r="E108" s="1" t="s">
@@ -4758,14 +4890,14 @@
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A109" s="39"/>
+      <c r="A109" s="38"/>
       <c r="B109" s="12" t="s">
         <v>144</v>
       </c>
       <c r="C109" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="D109" s="31" t="s">
+      <c r="D109" s="29" t="s">
         <v>86</v>
       </c>
       <c r="E109" s="1" t="s">
@@ -4776,14 +4908,14 @@
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A110" s="39"/>
+      <c r="A110" s="38"/>
       <c r="B110" s="12" t="s">
         <v>145</v>
       </c>
       <c r="C110" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="D110" s="31" t="s">
+      <c r="D110" s="29" t="s">
         <v>89</v>
       </c>
       <c r="E110" s="1" t="s">
@@ -4794,14 +4926,14 @@
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A111" s="39"/>
+      <c r="A111" s="38"/>
       <c r="B111" s="12" t="s">
         <v>146</v>
       </c>
       <c r="C111" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="D111" s="31" t="s">
+      <c r="D111" s="29" t="s">
         <v>92</v>
       </c>
       <c r="E111" s="1" t="s">
@@ -4812,14 +4944,14 @@
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A112" s="39"/>
+      <c r="A112" s="38"/>
       <c r="B112" s="12" t="s">
         <v>147</v>
       </c>
       <c r="C112" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="D112" s="31" t="s">
+      <c r="D112" s="29" t="s">
         <v>95</v>
       </c>
       <c r="E112" s="1" t="s">
@@ -4830,14 +4962,14 @@
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A113" s="39"/>
+      <c r="A113" s="38"/>
       <c r="B113" s="12" t="s">
         <v>148</v>
       </c>
       <c r="C113" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="D113" s="31" t="s">
+      <c r="D113" s="29" t="s">
         <v>98</v>
       </c>
       <c r="E113" s="1" t="s">
@@ -4848,14 +4980,14 @@
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A114" s="39"/>
+      <c r="A114" s="38"/>
       <c r="B114" s="12" t="s">
         <v>141</v>
       </c>
       <c r="C114" s="1" t="s">
         <v>279</v>
       </c>
-      <c r="D114" s="31" t="s">
+      <c r="D114" s="29" t="s">
         <v>101</v>
       </c>
       <c r="E114" s="1" t="s">
@@ -4866,14 +4998,14 @@
       </c>
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A115" s="39"/>
+      <c r="A115" s="38"/>
       <c r="B115" s="12" t="s">
         <v>138</v>
       </c>
       <c r="C115" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="D115" s="31" t="s">
+      <c r="D115" s="29" t="s">
         <v>104</v>
       </c>
       <c r="E115" s="1" t="s">
@@ -4884,14 +5016,14 @@
       </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A116" s="39"/>
+      <c r="A116" s="38"/>
       <c r="B116" s="12" t="s">
         <v>162</v>
       </c>
       <c r="C116" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D116" s="31" t="s">
+      <c r="D116" s="29" t="s">
         <v>35</v>
       </c>
       <c r="E116" s="1" t="s">
@@ -4902,14 +5034,14 @@
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A117" s="39"/>
+      <c r="A117" s="38"/>
       <c r="B117" s="12" t="s">
         <v>149</v>
       </c>
       <c r="C117" s="1" t="s">
         <v>283</v>
       </c>
-      <c r="D117" s="31" t="s">
+      <c r="D117" s="29" t="s">
         <v>107</v>
       </c>
       <c r="E117" s="1" t="s">
@@ -4920,14 +5052,14 @@
       </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A118" s="39"/>
+      <c r="A118" s="38"/>
       <c r="B118" s="12" t="s">
         <v>150</v>
       </c>
       <c r="C118" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="D118" s="31" t="s">
+      <c r="D118" s="29" t="s">
         <v>110</v>
       </c>
       <c r="E118" s="1" t="s">
@@ -4938,14 +5070,14 @@
       </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A119" s="39"/>
+      <c r="A119" s="38"/>
       <c r="B119" s="12" t="s">
         <v>138</v>
       </c>
       <c r="C119" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="D119" s="31" t="s">
+      <c r="D119" s="29" t="s">
         <v>113</v>
       </c>
       <c r="E119" s="1" t="s">
@@ -4956,14 +5088,14 @@
       </c>
     </row>
     <row r="120" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A120" s="39"/>
+      <c r="A120" s="38"/>
       <c r="B120" s="12" t="s">
         <v>163</v>
       </c>
       <c r="C120" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D120" s="31" t="s">
+      <c r="D120" s="29" t="s">
         <v>35</v>
       </c>
       <c r="E120" s="1" t="s">
@@ -4974,14 +5106,14 @@
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A121" s="39"/>
+      <c r="A121" s="38"/>
       <c r="B121" s="12" t="s">
         <v>151</v>
       </c>
       <c r="C121" s="1" t="s">
         <v>289</v>
       </c>
-      <c r="D121" s="31" t="s">
+      <c r="D121" s="29" t="s">
         <v>116</v>
       </c>
       <c r="E121" s="1" t="s">
@@ -4992,14 +5124,14 @@
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A122" s="39"/>
+      <c r="A122" s="38"/>
       <c r="B122" s="12" t="s">
         <v>152</v>
       </c>
       <c r="C122" s="1" t="s">
         <v>291</v>
       </c>
-      <c r="D122" s="31" t="s">
+      <c r="D122" s="29" t="s">
         <v>119</v>
       </c>
       <c r="E122" s="1" t="s">
@@ -5010,14 +5142,14 @@
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A123" s="39"/>
+      <c r="A123" s="38"/>
       <c r="B123" s="12" t="s">
         <v>153</v>
       </c>
       <c r="C123" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="D123" s="31" t="s">
+      <c r="D123" s="29" t="s">
         <v>122</v>
       </c>
       <c r="E123" s="1" t="s">
@@ -5028,20 +5160,20 @@
       </c>
     </row>
     <row r="124" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A124" s="40"/>
-      <c r="B124" s="32" t="s">
+      <c r="A124" s="39"/>
+      <c r="B124" s="30" t="s">
         <v>154</v>
       </c>
-      <c r="C124" s="33" t="s">
+      <c r="C124" s="31" t="s">
         <v>295</v>
       </c>
-      <c r="D124" s="34" t="s">
+      <c r="D124" s="32" t="s">
         <v>125</v>
       </c>
-      <c r="E124" s="33" t="s">
-        <v>35</v>
-      </c>
-      <c r="F124" s="33" t="s">
+      <c r="E124" s="31" t="s">
+        <v>35</v>
+      </c>
+      <c r="F124" s="31" t="s">
         <v>296</v>
       </c>
     </row>
@@ -5118,11 +5250,13 @@
       <c r="I133" s="12"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="6">
     <mergeCell ref="C3:F3"/>
     <mergeCell ref="A5:A44"/>
     <mergeCell ref="A45:A84"/>
     <mergeCell ref="A85:A124"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:B4"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5151,7 +5285,7 @@
         <v>456</v>
       </c>
       <c r="C1" s="2"/>
-      <c r="D1" s="30"/>
+      <c r="D1" s="28"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
@@ -5160,25 +5294,25 @@
     </row>
     <row r="2" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:9" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="27" t="s">
+      <c r="A3" s="40" t="s">
         <v>128</v>
       </c>
-      <c r="B3" s="27" t="s">
+      <c r="B3" s="40" t="s">
         <v>304</v>
       </c>
-      <c r="C3" s="37" t="s">
+      <c r="C3" s="36" t="s">
         <v>305</v>
       </c>
-      <c r="D3" s="37"/>
-      <c r="E3" s="37"/>
-      <c r="F3" s="37"/>
+      <c r="D3" s="36"/>
+      <c r="E3" s="36"/>
+      <c r="F3" s="36"/>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
     </row>
     <row r="4" spans="1:9" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="28"/>
-      <c r="B4" s="28"/>
+      <c r="A4" s="41"/>
+      <c r="B4" s="41"/>
       <c r="C4" s="6" t="s">
         <v>129</v>
       </c>
@@ -5196,7 +5330,7 @@
       <c r="I4" s="2"/>
     </row>
     <row r="5" spans="1:9" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="38" t="s">
+      <c r="A5" s="37" t="s">
         <v>157</v>
       </c>
       <c r="B5" s="9" t="s">
@@ -5205,7 +5339,7 @@
       <c r="C5" s="2" t="s">
         <v>307</v>
       </c>
-      <c r="D5" s="29" t="s">
+      <c r="D5" s="27" t="s">
         <v>308</v>
       </c>
       <c r="E5" s="2"/>
@@ -5217,7 +5351,7 @@
       <c r="I5" s="2"/>
     </row>
     <row r="6" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="39"/>
+      <c r="A6" s="38"/>
       <c r="B6" s="12" t="s">
         <v>167</v>
       </c>
@@ -5235,7 +5369,7 @@
       </c>
     </row>
     <row r="7" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="39"/>
+      <c r="A7" s="38"/>
       <c r="B7" s="12" t="s">
         <v>131</v>
       </c>
@@ -5253,7 +5387,7 @@
       </c>
     </row>
     <row r="8" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="39"/>
+      <c r="A8" s="38"/>
       <c r="B8" s="12" t="s">
         <v>168</v>
       </c>
@@ -5271,7 +5405,7 @@
       </c>
     </row>
     <row r="9" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="39"/>
+      <c r="A9" s="38"/>
       <c r="B9" s="12" t="s">
         <v>131</v>
       </c>
@@ -5289,7 +5423,7 @@
       </c>
     </row>
     <row r="10" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="39"/>
+      <c r="A10" s="38"/>
       <c r="B10" s="12" t="s">
         <v>297</v>
       </c>
@@ -5307,7 +5441,7 @@
       </c>
     </row>
     <row r="11" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="39"/>
+      <c r="A11" s="38"/>
       <c r="B11" s="12" t="s">
         <v>131</v>
       </c>
@@ -5325,7 +5459,7 @@
       </c>
     </row>
     <row r="12" spans="1:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="39"/>
+      <c r="A12" s="38"/>
       <c r="B12" s="12" t="s">
         <v>160</v>
       </c>
@@ -5343,7 +5477,7 @@
       </c>
     </row>
     <row r="13" spans="1:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="39"/>
+      <c r="A13" s="38"/>
       <c r="B13" s="12" t="s">
         <v>141</v>
       </c>
@@ -5361,7 +5495,7 @@
       </c>
     </row>
     <row r="14" spans="1:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="39"/>
+      <c r="A14" s="38"/>
       <c r="B14" s="12" t="s">
         <v>142</v>
       </c>
@@ -5379,7 +5513,7 @@
       </c>
     </row>
     <row r="15" spans="1:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="39"/>
+      <c r="A15" s="38"/>
       <c r="B15" s="12" t="s">
         <v>143</v>
       </c>
@@ -5397,7 +5531,7 @@
       </c>
     </row>
     <row r="16" spans="1:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="39"/>
+      <c r="A16" s="38"/>
       <c r="B16" s="12" t="s">
         <v>138</v>
       </c>
@@ -5415,7 +5549,7 @@
       </c>
     </row>
     <row r="17" spans="1:6" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="39"/>
+      <c r="A17" s="38"/>
       <c r="B17" s="12" t="s">
         <v>161</v>
       </c>
@@ -5433,7 +5567,7 @@
       </c>
     </row>
     <row r="18" spans="1:6" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="39"/>
+      <c r="A18" s="38"/>
       <c r="B18" s="12" t="s">
         <v>144</v>
       </c>
@@ -5451,7 +5585,7 @@
       </c>
     </row>
     <row r="19" spans="1:6" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="39"/>
+      <c r="A19" s="38"/>
       <c r="B19" s="12" t="s">
         <v>145</v>
       </c>
@@ -5469,7 +5603,7 @@
       </c>
     </row>
     <row r="20" spans="1:6" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="39"/>
+      <c r="A20" s="38"/>
       <c r="B20" s="12" t="s">
         <v>146</v>
       </c>
@@ -5487,7 +5621,7 @@
       </c>
     </row>
     <row r="21" spans="1:6" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="39"/>
+      <c r="A21" s="38"/>
       <c r="B21" s="12" t="s">
         <v>147</v>
       </c>
@@ -5505,7 +5639,7 @@
       </c>
     </row>
     <row r="22" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="39"/>
+      <c r="A22" s="38"/>
       <c r="B22" s="12" t="s">
         <v>148</v>
       </c>
@@ -5523,7 +5657,7 @@
       </c>
     </row>
     <row r="23" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="39"/>
+      <c r="A23" s="38"/>
       <c r="B23" s="12" t="s">
         <v>141</v>
       </c>
@@ -5541,7 +5675,7 @@
       </c>
     </row>
     <row r="24" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="39"/>
+      <c r="A24" s="38"/>
       <c r="B24" s="12" t="s">
         <v>138</v>
       </c>
@@ -5559,7 +5693,7 @@
       </c>
     </row>
     <row r="25" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="39"/>
+      <c r="A25" s="38"/>
       <c r="B25" s="12" t="s">
         <v>162</v>
       </c>
@@ -5577,7 +5711,7 @@
       </c>
     </row>
     <row r="26" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="39"/>
+      <c r="A26" s="38"/>
       <c r="B26" s="12" t="s">
         <v>149</v>
       </c>
@@ -5595,7 +5729,7 @@
       </c>
     </row>
     <row r="27" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="39"/>
+      <c r="A27" s="38"/>
       <c r="B27" s="12" t="s">
         <v>150</v>
       </c>
@@ -5613,7 +5747,7 @@
       </c>
     </row>
     <row r="28" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="39"/>
+      <c r="A28" s="38"/>
       <c r="B28" s="12" t="s">
         <v>138</v>
       </c>
@@ -5631,7 +5765,7 @@
       </c>
     </row>
     <row r="29" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="39"/>
+      <c r="A29" s="38"/>
       <c r="B29" s="12" t="s">
         <v>163</v>
       </c>
@@ -5649,7 +5783,7 @@
       </c>
     </row>
     <row r="30" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="39"/>
+      <c r="A30" s="38"/>
       <c r="B30" s="12" t="s">
         <v>151</v>
       </c>
@@ -5667,7 +5801,7 @@
       </c>
     </row>
     <row r="31" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="39"/>
+      <c r="A31" s="38"/>
       <c r="B31" s="12" t="s">
         <v>152</v>
       </c>
@@ -5685,7 +5819,7 @@
       </c>
     </row>
     <row r="32" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="39"/>
+      <c r="A32" s="38"/>
       <c r="B32" s="12" t="s">
         <v>153</v>
       </c>
@@ -5703,7 +5837,7 @@
       </c>
     </row>
     <row r="33" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="39"/>
+      <c r="A33" s="38"/>
       <c r="B33" s="12" t="s">
         <v>154</v>
       </c>
@@ -5721,7 +5855,7 @@
       </c>
     </row>
     <row r="34" spans="1:9" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A34" s="39" t="s">
+      <c r="A34" s="38" t="s">
         <v>169</v>
       </c>
       <c r="B34" s="9" t="s">
@@ -5730,7 +5864,7 @@
       <c r="C34" s="2" t="s">
         <v>373</v>
       </c>
-      <c r="D34" s="30" t="s">
+      <c r="D34" s="28" t="s">
         <v>308</v>
       </c>
       <c r="E34" s="2"/>
@@ -5742,7 +5876,7 @@
       <c r="I34" s="2"/>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A35" s="39"/>
+      <c r="A35" s="38"/>
       <c r="B35" s="12" t="s">
         <v>167</v>
       </c>
@@ -5760,7 +5894,7 @@
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" s="39"/>
+      <c r="A36" s="38"/>
       <c r="B36" s="12" t="s">
         <v>131</v>
       </c>
@@ -5778,7 +5912,7 @@
       </c>
     </row>
     <row r="37" spans="1:9" ht="18" x14ac:dyDescent="0.25">
-      <c r="A37" s="39"/>
+      <c r="A37" s="38"/>
       <c r="B37" s="12" t="s">
         <v>168</v>
       </c>
@@ -5796,7 +5930,7 @@
       </c>
     </row>
     <row r="38" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="39"/>
+      <c r="A38" s="38"/>
       <c r="B38" s="12" t="s">
         <v>131</v>
       </c>
@@ -5814,7 +5948,7 @@
       </c>
     </row>
     <row r="39" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="39"/>
+      <c r="A39" s="38"/>
       <c r="B39" s="12" t="s">
         <v>297</v>
       </c>
@@ -5832,7 +5966,7 @@
       </c>
     </row>
     <row r="40" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="39"/>
+      <c r="A40" s="38"/>
       <c r="B40" s="12" t="s">
         <v>131</v>
       </c>
@@ -5850,7 +5984,7 @@
       </c>
     </row>
     <row r="41" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="39"/>
+      <c r="A41" s="38"/>
       <c r="B41" s="12" t="s">
         <v>160</v>
       </c>
@@ -5868,7 +6002,7 @@
       </c>
     </row>
     <row r="42" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="39"/>
+      <c r="A42" s="38"/>
       <c r="B42" s="12" t="s">
         <v>141</v>
       </c>
@@ -5886,7 +6020,7 @@
       </c>
     </row>
     <row r="43" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="39"/>
+      <c r="A43" s="38"/>
       <c r="B43" s="12" t="s">
         <v>142</v>
       </c>
@@ -5904,7 +6038,7 @@
       </c>
     </row>
     <row r="44" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="39"/>
+      <c r="A44" s="38"/>
       <c r="B44" s="12" t="s">
         <v>143</v>
       </c>
@@ -5922,7 +6056,7 @@
       </c>
     </row>
     <row r="45" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="39"/>
+      <c r="A45" s="38"/>
       <c r="B45" s="12" t="s">
         <v>138</v>
       </c>
@@ -5940,7 +6074,7 @@
       </c>
     </row>
     <row r="46" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="39"/>
+      <c r="A46" s="38"/>
       <c r="B46" s="12" t="s">
         <v>161</v>
       </c>
@@ -5958,7 +6092,7 @@
       </c>
     </row>
     <row r="47" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="39"/>
+      <c r="A47" s="38"/>
       <c r="B47" s="12" t="s">
         <v>144</v>
       </c>
@@ -5976,7 +6110,7 @@
       </c>
     </row>
     <row r="48" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="39"/>
+      <c r="A48" s="38"/>
       <c r="B48" s="12" t="s">
         <v>145</v>
       </c>
@@ -5994,7 +6128,7 @@
       </c>
     </row>
     <row r="49" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="39"/>
+      <c r="A49" s="38"/>
       <c r="B49" s="12" t="s">
         <v>146</v>
       </c>
@@ -6012,7 +6146,7 @@
       </c>
     </row>
     <row r="50" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="39"/>
+      <c r="A50" s="38"/>
       <c r="B50" s="12" t="s">
         <v>147</v>
       </c>
@@ -6030,7 +6164,7 @@
       </c>
     </row>
     <row r="51" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="39"/>
+      <c r="A51" s="38"/>
       <c r="B51" s="12" t="s">
         <v>148</v>
       </c>
@@ -6048,7 +6182,7 @@
       </c>
     </row>
     <row r="52" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="39"/>
+      <c r="A52" s="38"/>
       <c r="B52" s="12" t="s">
         <v>141</v>
       </c>
@@ -6066,7 +6200,7 @@
       </c>
     </row>
     <row r="53" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="39"/>
+      <c r="A53" s="38"/>
       <c r="B53" s="12" t="s">
         <v>138</v>
       </c>
@@ -6084,7 +6218,7 @@
       </c>
     </row>
     <row r="54" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="39"/>
+      <c r="A54" s="38"/>
       <c r="B54" s="12" t="s">
         <v>162</v>
       </c>
@@ -6102,7 +6236,7 @@
       </c>
     </row>
     <row r="55" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="39"/>
+      <c r="A55" s="38"/>
       <c r="B55" s="12" t="s">
         <v>149</v>
       </c>
@@ -6120,7 +6254,7 @@
       </c>
     </row>
     <row r="56" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="39"/>
+      <c r="A56" s="38"/>
       <c r="B56" s="12" t="s">
         <v>150</v>
       </c>
@@ -6138,7 +6272,7 @@
       </c>
     </row>
     <row r="57" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="39"/>
+      <c r="A57" s="38"/>
       <c r="B57" s="12" t="s">
         <v>138</v>
       </c>
@@ -6156,7 +6290,7 @@
       </c>
     </row>
     <row r="58" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="39"/>
+      <c r="A58" s="38"/>
       <c r="B58" s="12" t="s">
         <v>163</v>
       </c>
@@ -6174,7 +6308,7 @@
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A59" s="39"/>
+      <c r="A59" s="38"/>
       <c r="B59" s="12" t="s">
         <v>151</v>
       </c>
@@ -6192,7 +6326,7 @@
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A60" s="39"/>
+      <c r="A60" s="38"/>
       <c r="B60" s="12" t="s">
         <v>152</v>
       </c>
@@ -6210,7 +6344,7 @@
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A61" s="39"/>
+      <c r="A61" s="38"/>
       <c r="B61" s="12" t="s">
         <v>153</v>
       </c>
@@ -6228,7 +6362,7 @@
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A62" s="39"/>
+      <c r="A62" s="38"/>
       <c r="B62" s="12" t="s">
         <v>154</v>
       </c>
@@ -6246,7 +6380,7 @@
       </c>
     </row>
     <row r="63" spans="1:9" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A63" s="39" t="s">
+      <c r="A63" s="38" t="s">
         <v>236</v>
       </c>
       <c r="B63" s="9" t="s">
@@ -6255,7 +6389,7 @@
       <c r="C63" s="2" t="s">
         <v>415</v>
       </c>
-      <c r="D63" s="29" t="s">
+      <c r="D63" s="27" t="s">
         <v>308</v>
       </c>
       <c r="E63" s="2"/>
@@ -6267,14 +6401,14 @@
       <c r="I63" s="2"/>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A64" s="39"/>
+      <c r="A64" s="38"/>
       <c r="B64" s="12" t="s">
         <v>167</v>
       </c>
       <c r="C64" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D64" s="31" t="s">
+      <c r="D64" s="29" t="s">
         <v>35</v>
       </c>
       <c r="E64" s="1" t="s">
@@ -6285,14 +6419,14 @@
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A65" s="39"/>
+      <c r="A65" s="38"/>
       <c r="B65" s="12" t="s">
         <v>131</v>
       </c>
       <c r="C65" s="1" t="s">
         <v>417</v>
       </c>
-      <c r="D65" s="31" t="s">
+      <c r="D65" s="29" t="s">
         <v>311</v>
       </c>
       <c r="E65" s="1" t="s">
@@ -6303,14 +6437,14 @@
       </c>
     </row>
     <row r="66" spans="1:6" ht="18" x14ac:dyDescent="0.25">
-      <c r="A66" s="39"/>
+      <c r="A66" s="38"/>
       <c r="B66" s="12" t="s">
         <v>168</v>
       </c>
       <c r="C66" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D66" s="31" t="s">
+      <c r="D66" s="29" t="s">
         <v>35</v>
       </c>
       <c r="E66" s="1" t="s">
@@ -6321,14 +6455,14 @@
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A67" s="39"/>
+      <c r="A67" s="38"/>
       <c r="B67" s="12" t="s">
         <v>131</v>
       </c>
       <c r="C67" s="1" t="s">
         <v>418</v>
       </c>
-      <c r="D67" s="31" t="s">
+      <c r="D67" s="29" t="s">
         <v>314</v>
       </c>
       <c r="E67" s="1" t="s">
@@ -6339,14 +6473,14 @@
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A68" s="39"/>
+      <c r="A68" s="38"/>
       <c r="B68" s="12" t="s">
         <v>297</v>
       </c>
       <c r="C68" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D68" s="31" t="s">
+      <c r="D68" s="29" t="s">
         <v>35</v>
       </c>
       <c r="E68" s="1" t="s">
@@ -6357,14 +6491,14 @@
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A69" s="39"/>
+      <c r="A69" s="38"/>
       <c r="B69" s="12" t="s">
         <v>131</v>
       </c>
       <c r="C69" s="1" t="s">
         <v>419</v>
       </c>
-      <c r="D69" s="31" t="s">
+      <c r="D69" s="29" t="s">
         <v>317</v>
       </c>
       <c r="E69" s="1" t="s">
@@ -6375,14 +6509,14 @@
       </c>
     </row>
     <row r="70" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="39"/>
+      <c r="A70" s="38"/>
       <c r="B70" s="12" t="s">
         <v>160</v>
       </c>
       <c r="C70" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D70" s="31" t="s">
+      <c r="D70" s="29" t="s">
         <v>35</v>
       </c>
       <c r="E70" s="1" t="s">
@@ -6393,14 +6527,14 @@
       </c>
     </row>
     <row r="71" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="39"/>
+      <c r="A71" s="38"/>
       <c r="B71" s="12" t="s">
         <v>141</v>
       </c>
       <c r="C71" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="D71" s="31" t="s">
+      <c r="D71" s="29" t="s">
         <v>320</v>
       </c>
       <c r="E71" s="1" t="s">
@@ -6411,14 +6545,14 @@
       </c>
     </row>
     <row r="72" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="39"/>
+      <c r="A72" s="38"/>
       <c r="B72" s="12" t="s">
         <v>142</v>
       </c>
       <c r="C72" s="1" t="s">
         <v>422</v>
       </c>
-      <c r="D72" s="31" t="s">
+      <c r="D72" s="29" t="s">
         <v>323</v>
       </c>
       <c r="E72" s="1" t="s">
@@ -6429,14 +6563,14 @@
       </c>
     </row>
     <row r="73" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="39"/>
+      <c r="A73" s="38"/>
       <c r="B73" s="12" t="s">
         <v>143</v>
       </c>
       <c r="C73" s="1" t="s">
         <v>424</v>
       </c>
-      <c r="D73" s="31" t="s">
+      <c r="D73" s="29" t="s">
         <v>326</v>
       </c>
       <c r="E73" s="1" t="s">
@@ -6447,14 +6581,14 @@
       </c>
     </row>
     <row r="74" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="39"/>
+      <c r="A74" s="38"/>
       <c r="B74" s="12" t="s">
         <v>138</v>
       </c>
       <c r="C74" s="1" t="s">
         <v>426</v>
       </c>
-      <c r="D74" s="31" t="s">
+      <c r="D74" s="29" t="s">
         <v>329</v>
       </c>
       <c r="E74" s="1" t="s">
@@ -6465,14 +6599,14 @@
       </c>
     </row>
     <row r="75" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="39"/>
+      <c r="A75" s="38"/>
       <c r="B75" s="12" t="s">
         <v>161</v>
       </c>
       <c r="C75" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D75" s="31" t="s">
+      <c r="D75" s="29" t="s">
         <v>35</v>
       </c>
       <c r="E75" s="1" t="s">
@@ -6483,14 +6617,14 @@
       </c>
     </row>
     <row r="76" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="39"/>
+      <c r="A76" s="38"/>
       <c r="B76" s="12" t="s">
         <v>144</v>
       </c>
       <c r="C76" s="1" t="s">
         <v>429</v>
       </c>
-      <c r="D76" s="31" t="s">
+      <c r="D76" s="29" t="s">
         <v>333</v>
       </c>
       <c r="E76" s="1" t="s">
@@ -6501,14 +6635,14 @@
       </c>
     </row>
     <row r="77" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="39"/>
+      <c r="A77" s="38"/>
       <c r="B77" s="12" t="s">
         <v>145</v>
       </c>
       <c r="C77" s="1" t="s">
         <v>431</v>
       </c>
-      <c r="D77" s="31" t="s">
+      <c r="D77" s="29" t="s">
         <v>336</v>
       </c>
       <c r="E77" s="1" t="s">
@@ -6519,14 +6653,14 @@
       </c>
     </row>
     <row r="78" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="39"/>
+      <c r="A78" s="38"/>
       <c r="B78" s="12" t="s">
         <v>146</v>
       </c>
       <c r="C78" s="1" t="s">
         <v>433</v>
       </c>
-      <c r="D78" s="31" t="s">
+      <c r="D78" s="29" t="s">
         <v>339</v>
       </c>
       <c r="E78" s="1" t="s">
@@ -6537,14 +6671,14 @@
       </c>
     </row>
     <row r="79" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="39"/>
+      <c r="A79" s="38"/>
       <c r="B79" s="12" t="s">
         <v>147</v>
       </c>
       <c r="C79" s="1" t="s">
         <v>435</v>
       </c>
-      <c r="D79" s="31" t="s">
+      <c r="D79" s="29" t="s">
         <v>342</v>
       </c>
       <c r="E79" s="1" t="s">
@@ -6555,14 +6689,14 @@
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A80" s="39"/>
+      <c r="A80" s="38"/>
       <c r="B80" s="12" t="s">
         <v>148</v>
       </c>
       <c r="C80" s="1" t="s">
         <v>437</v>
       </c>
-      <c r="D80" s="31" t="s">
+      <c r="D80" s="29" t="s">
         <v>345</v>
       </c>
       <c r="E80" s="1" t="s">
@@ -6573,14 +6707,14 @@
       </c>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A81" s="39"/>
+      <c r="A81" s="38"/>
       <c r="B81" s="12" t="s">
         <v>141</v>
       </c>
       <c r="C81" s="1" t="s">
         <v>439</v>
       </c>
-      <c r="D81" s="31" t="s">
+      <c r="D81" s="29" t="s">
         <v>348</v>
       </c>
       <c r="E81" s="1" t="s">
@@ -6591,14 +6725,14 @@
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A82" s="39"/>
+      <c r="A82" s="38"/>
       <c r="B82" s="12" t="s">
         <v>138</v>
       </c>
       <c r="C82" s="1" t="s">
         <v>441</v>
       </c>
-      <c r="D82" s="31" t="s">
+      <c r="D82" s="29" t="s">
         <v>351</v>
       </c>
       <c r="E82" s="1" t="s">
@@ -6609,14 +6743,14 @@
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A83" s="39"/>
+      <c r="A83" s="38"/>
       <c r="B83" s="12" t="s">
         <v>162</v>
       </c>
       <c r="C83" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D83" s="31" t="s">
+      <c r="D83" s="29" t="s">
         <v>35</v>
       </c>
       <c r="E83" s="1" t="s">
@@ -6627,14 +6761,14 @@
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A84" s="39"/>
+      <c r="A84" s="38"/>
       <c r="B84" s="12" t="s">
         <v>149</v>
       </c>
       <c r="C84" s="1" t="s">
         <v>442</v>
       </c>
-      <c r="D84" s="31" t="s">
+      <c r="D84" s="29" t="s">
         <v>354</v>
       </c>
       <c r="E84" s="1" t="s">
@@ -6645,14 +6779,14 @@
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A85" s="39"/>
+      <c r="A85" s="38"/>
       <c r="B85" s="12" t="s">
         <v>150</v>
       </c>
       <c r="C85" s="1" t="s">
         <v>444</v>
       </c>
-      <c r="D85" s="31" t="s">
+      <c r="D85" s="29" t="s">
         <v>357</v>
       </c>
       <c r="E85" s="1" t="s">
@@ -6663,14 +6797,14 @@
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A86" s="39"/>
+      <c r="A86" s="38"/>
       <c r="B86" s="12" t="s">
         <v>138</v>
       </c>
       <c r="C86" s="1" t="s">
         <v>359</v>
       </c>
-      <c r="D86" s="31" t="s">
+      <c r="D86" s="29" t="s">
         <v>359</v>
       </c>
       <c r="E86" s="1" t="s">
@@ -6681,14 +6815,14 @@
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A87" s="39"/>
+      <c r="A87" s="38"/>
       <c r="B87" s="12" t="s">
         <v>163</v>
       </c>
       <c r="C87" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D87" s="31" t="s">
+      <c r="D87" s="29" t="s">
         <v>35</v>
       </c>
       <c r="E87" s="1" t="s">
@@ -6699,14 +6833,14 @@
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A88" s="39"/>
+      <c r="A88" s="38"/>
       <c r="B88" s="12" t="s">
         <v>151</v>
       </c>
       <c r="C88" s="1" t="s">
         <v>447</v>
       </c>
-      <c r="D88" s="31" t="s">
+      <c r="D88" s="29" t="s">
         <v>362</v>
       </c>
       <c r="E88" s="1" t="s">
@@ -6717,14 +6851,14 @@
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A89" s="39"/>
+      <c r="A89" s="38"/>
       <c r="B89" s="12" t="s">
         <v>152</v>
       </c>
       <c r="C89" s="1" t="s">
         <v>449</v>
       </c>
-      <c r="D89" s="31" t="s">
+      <c r="D89" s="29" t="s">
         <v>365</v>
       </c>
       <c r="E89" s="1" t="s">
@@ -6735,14 +6869,14 @@
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A90" s="39"/>
+      <c r="A90" s="38"/>
       <c r="B90" s="12" t="s">
         <v>153</v>
       </c>
       <c r="C90" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="D90" s="31" t="s">
+      <c r="D90" s="29" t="s">
         <v>368</v>
       </c>
       <c r="E90" s="1" t="s">
@@ -6753,20 +6887,20 @@
       </c>
     </row>
     <row r="91" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A91" s="40"/>
-      <c r="B91" s="32" t="s">
+      <c r="A91" s="39"/>
+      <c r="B91" s="30" t="s">
         <v>154</v>
       </c>
-      <c r="C91" s="33" t="s">
+      <c r="C91" s="31" t="s">
         <v>453</v>
       </c>
-      <c r="D91" s="34" t="s">
+      <c r="D91" s="32" t="s">
         <v>371</v>
       </c>
-      <c r="E91" s="33" t="s">
-        <v>35</v>
-      </c>
-      <c r="F91" s="33" t="s">
+      <c r="E91" s="31" t="s">
+        <v>35</v>
+      </c>
+      <c r="F91" s="31" t="s">
         <v>454</v>
       </c>
     </row>
@@ -6852,11 +6986,13 @@
       <c r="I101" s="12"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="6">
     <mergeCell ref="C3:F3"/>
     <mergeCell ref="A5:A33"/>
     <mergeCell ref="A34:A62"/>
     <mergeCell ref="A63:A91"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:B4"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
docs(output): :memo: Update Table S5 for presenting the Tracy-Wisdom statistics
</commit_message>
<xml_diff>
--- a/output/Tables/mmc1.xlsx
+++ b/output/Tables/mmc1.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\luzh29\Library\Projects\WGS_GWAS_and_MR\output\Tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88D8432C-2C63-4990-86F5-5E2B9B7EE633}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB9A7903-D320-40C2-B0A2-8E0E1B818E92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="16440" windowHeight="28320" tabRatio="692" activeTab="1" xr2:uid="{B1B36BAE-942B-7148-AF58-4A36D0B24BEE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="692" activeTab="4" xr2:uid="{B1B36BAE-942B-7148-AF58-4A36D0B24BEE}"/>
   </bookViews>
   <sheets>
     <sheet name="Table S1" sheetId="49" r:id="rId1"/>
     <sheet name="Table S2" sheetId="53" r:id="rId2"/>
     <sheet name="Table S3" sheetId="51" r:id="rId3"/>
     <sheet name="Table S4" sheetId="52" r:id="rId4"/>
+    <sheet name="Table S5" sheetId="54" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1154" uniqueCount="501">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1491" uniqueCount="511">
   <si>
     <t>Disease</t>
   </si>
@@ -1724,6 +1725,45 @@
   </si>
   <si>
     <t>Cancer diagnosed by doctor | Instance 0-3; Coding Meaning: https://biobank.ndph.ox.ac.uk/showcase/field.cgi?id=2453</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Principal components</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>eigenvalue</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>difference</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>twstat</t>
+  </si>
+  <si>
+    <t>NA</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Table S5. Tracy-Widom statistics of top 30 principal components for the UKBB cohorts, by phenotypes and ethnicities.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>twstat: Tracy-Widom statistic.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>effect n*</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>*effect n is the effective number of independent markers/samples.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>NA: not available.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -6999,16 +7039,1903 @@
 </worksheet>
 </file>
 
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EC88E03-DBCE-4AE3-86E5-68AC9CDB987B}">
+  <dimension ref="A1:J104"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="25.875" style="12" customWidth="1"/>
+    <col min="2" max="2" width="27" style="10" customWidth="1"/>
+    <col min="3" max="3" width="20.5" style="1" customWidth="1"/>
+    <col min="4" max="4" width="23.375" style="7" customWidth="1"/>
+    <col min="5" max="5" width="19.125" style="7" customWidth="1"/>
+    <col min="6" max="6" width="11.625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="23.5" style="1" customWidth="1"/>
+    <col min="8" max="8" width="34.5" style="1" customWidth="1"/>
+    <col min="9" max="9" width="31.75" style="1" customWidth="1"/>
+    <col min="10" max="10" width="22.875" style="1" customWidth="1"/>
+    <col min="11" max="16384" width="11" style="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>506</v>
+      </c>
+      <c r="B1" s="16"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+    </row>
+    <row r="2" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="1:10" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="B3" s="40" t="s">
+        <v>501</v>
+      </c>
+      <c r="C3" s="36" t="s">
+        <v>305</v>
+      </c>
+      <c r="D3" s="36"/>
+      <c r="E3" s="36"/>
+      <c r="F3" s="36"/>
+      <c r="G3" s="36"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+    </row>
+    <row r="4" spans="1:10" s="9" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="41"/>
+      <c r="B4" s="41"/>
+      <c r="C4" s="6" t="s">
+        <v>502</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>503</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>504</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>508</v>
+      </c>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="37" t="s">
+        <v>157</v>
+      </c>
+      <c r="B5" s="10">
+        <v>1</v>
+      </c>
+      <c r="C5" s="1">
+        <v>34.405000000000001</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="E5" s="1">
+        <v>11.81</v>
+      </c>
+      <c r="F5" s="1">
+        <v>1.3508300000000001E-13</v>
+      </c>
+      <c r="G5" s="1">
+        <v>60.408999999999999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="38"/>
+      <c r="B6" s="10">
+        <v>2</v>
+      </c>
+      <c r="C6" s="1">
+        <v>15.432</v>
+      </c>
+      <c r="D6" s="1">
+        <v>-18.972999999999999</v>
+      </c>
+      <c r="E6" s="1">
+        <v>13.997</v>
+      </c>
+      <c r="F6" s="1">
+        <v>5.0215200000000001E-17</v>
+      </c>
+      <c r="G6" s="1">
+        <v>301.08499999999998</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="38"/>
+      <c r="B7" s="10">
+        <v>3</v>
+      </c>
+      <c r="C7" s="1">
+        <v>12.2</v>
+      </c>
+      <c r="D7" s="1">
+        <v>-3.2320000000000002</v>
+      </c>
+      <c r="E7" s="1">
+        <v>20.241</v>
+      </c>
+      <c r="F7" s="1">
+        <v>2.8580900000000001E-28</v>
+      </c>
+      <c r="G7" s="1">
+        <v>732.77499999999998</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="38"/>
+      <c r="B8" s="10">
+        <v>4</v>
+      </c>
+      <c r="C8" s="1">
+        <v>7.6479999999999997</v>
+      </c>
+      <c r="D8" s="1">
+        <v>-4.5519999999999996</v>
+      </c>
+      <c r="E8" s="1">
+        <v>12.257999999999999</v>
+      </c>
+      <c r="F8" s="1">
+        <v>2.82331E-14</v>
+      </c>
+      <c r="G8" s="1">
+        <v>4352.2690000000002</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="38"/>
+      <c r="B9" s="10">
+        <v>5</v>
+      </c>
+      <c r="C9" s="1">
+        <v>7.4589999999999996</v>
+      </c>
+      <c r="D9" s="1">
+        <v>-0.189</v>
+      </c>
+      <c r="E9" s="1">
+        <v>19.318999999999999</v>
+      </c>
+      <c r="F9" s="1">
+        <v>1.7529999999999999E-26</v>
+      </c>
+      <c r="G9" s="1">
+        <v>7325.8649999999998</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="38"/>
+      <c r="B10" s="10">
+        <v>6</v>
+      </c>
+      <c r="C10" s="1">
+        <v>6.46</v>
+      </c>
+      <c r="D10" s="1">
+        <v>-0.999</v>
+      </c>
+      <c r="E10" s="1">
+        <v>10.804</v>
+      </c>
+      <c r="F10" s="1">
+        <v>4.0646999999999998E-12</v>
+      </c>
+      <c r="G10" s="1">
+        <v>24673.268</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="38"/>
+      <c r="B11" s="10">
+        <v>7</v>
+      </c>
+      <c r="C11" s="1">
+        <v>6.2450000000000001</v>
+      </c>
+      <c r="D11" s="1">
+        <v>-0.215</v>
+      </c>
+      <c r="E11" s="1">
+        <v>8.1549999999999994</v>
+      </c>
+      <c r="F11" s="1">
+        <v>1.5109400000000002E-8</v>
+      </c>
+      <c r="G11" s="1">
+        <v>39833.605000000003</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="38"/>
+      <c r="B12" s="10">
+        <v>8</v>
+      </c>
+      <c r="C12" s="1">
+        <v>6.0789999999999997</v>
+      </c>
+      <c r="D12" s="1">
+        <v>-0.16600000000000001</v>
+      </c>
+      <c r="E12" s="1">
+        <v>3.5979999999999999</v>
+      </c>
+      <c r="F12" s="1">
+        <v>5.1616399999999995E-4</v>
+      </c>
+      <c r="G12" s="1">
+        <v>57874.345999999998</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="38"/>
+      <c r="B13" s="10">
+        <v>9</v>
+      </c>
+      <c r="C13" s="1">
+        <v>6.0289999999999999</v>
+      </c>
+      <c r="D13" s="1">
+        <v>-0.05</v>
+      </c>
+      <c r="E13" s="1">
+        <v>3.3140000000000001</v>
+      </c>
+      <c r="F13" s="1">
+        <v>9.1978000000000003E-4</v>
+      </c>
+      <c r="G13" s="1">
+        <v>71139.604000000007</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="38"/>
+      <c r="B14" s="10">
+        <v>10</v>
+      </c>
+      <c r="C14" s="1">
+        <v>5.9409999999999998</v>
+      </c>
+      <c r="D14" s="1">
+        <v>-8.7999999999999995E-2</v>
+      </c>
+      <c r="E14" s="1">
+        <v>-0.58299999999999996</v>
+      </c>
+      <c r="F14" s="1">
+        <v>0.29766799999999999</v>
+      </c>
+      <c r="G14" s="1">
+        <v>87789.077000000005</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="38"/>
+      <c r="B15" s="10">
+        <v>11</v>
+      </c>
+      <c r="C15" s="1">
+        <v>5.915</v>
+      </c>
+      <c r="D15" s="1">
+        <v>-2.5999999999999999E-2</v>
+      </c>
+      <c r="E15" s="1">
+        <v>-1.0289999999999999</v>
+      </c>
+      <c r="F15" s="1">
+        <v>0.425182</v>
+      </c>
+      <c r="G15" s="1">
+        <v>96203.793999999994</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="38"/>
+      <c r="B16" s="10">
+        <v>12</v>
+      </c>
+      <c r="C16" s="1">
+        <v>5.8890000000000002</v>
+      </c>
+      <c r="D16" s="1">
+        <v>-2.5999999999999999E-2</v>
+      </c>
+      <c r="E16" s="1">
+        <v>-1.67</v>
+      </c>
+      <c r="F16" s="1">
+        <v>0.62729999999999997</v>
+      </c>
+      <c r="G16" s="1">
+        <v>104500.33900000001</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="38"/>
+      <c r="B17" s="10">
+        <v>13</v>
+      </c>
+      <c r="C17" s="1">
+        <v>5.8719999999999999</v>
+      </c>
+      <c r="D17" s="1">
+        <v>-1.7000000000000001E-2</v>
+      </c>
+      <c r="E17" s="1">
+        <v>-1.7110000000000001</v>
+      </c>
+      <c r="F17" s="1">
+        <v>0.64012100000000005</v>
+      </c>
+      <c r="G17" s="1">
+        <v>111706.451</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="38"/>
+      <c r="B18" s="10">
+        <v>14</v>
+      </c>
+      <c r="C18" s="1">
+        <v>5.8630000000000004</v>
+      </c>
+      <c r="D18" s="1">
+        <v>-8.9999999999999993E-3</v>
+      </c>
+      <c r="E18" s="1">
+        <v>-1.0289999999999999</v>
+      </c>
+      <c r="F18" s="1">
+        <v>0.42511199999999999</v>
+      </c>
+      <c r="G18" s="1">
+        <v>119533.844</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="38"/>
+      <c r="B19" s="10">
+        <v>15</v>
+      </c>
+      <c r="C19" s="1">
+        <v>5.8570000000000002</v>
+      </c>
+      <c r="D19" s="1">
+        <v>-6.0000000000000001E-3</v>
+      </c>
+      <c r="E19" s="1">
+        <v>0.16700000000000001</v>
+      </c>
+      <c r="F19" s="1">
+        <v>0.139735</v>
+      </c>
+      <c r="G19" s="1">
+        <v>131547.61199999999</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="38"/>
+      <c r="B20" s="10">
+        <v>16</v>
+      </c>
+      <c r="C20" s="1">
+        <v>5.8449999999999998</v>
+      </c>
+      <c r="D20" s="1">
+        <v>-1.2E-2</v>
+      </c>
+      <c r="E20" s="1">
+        <v>1.26</v>
+      </c>
+      <c r="F20" s="1">
+        <v>3.3467700000000003E-2</v>
+      </c>
+      <c r="G20" s="1">
+        <v>153990.29699999999</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="38"/>
+      <c r="B21" s="10">
+        <v>17</v>
+      </c>
+      <c r="C21" s="1">
+        <v>5.8250000000000002</v>
+      </c>
+      <c r="D21" s="1">
+        <v>-0.02</v>
+      </c>
+      <c r="E21" s="1">
+        <v>2.0430000000000001</v>
+      </c>
+      <c r="F21" s="1">
+        <v>9.6745500000000005E-3</v>
+      </c>
+      <c r="G21" s="1">
+        <v>195526.43400000001</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="38"/>
+      <c r="B22" s="10">
+        <v>18</v>
+      </c>
+      <c r="C22" s="1">
+        <v>5.7789999999999999</v>
+      </c>
+      <c r="D22" s="1">
+        <v>-4.5999999999999999E-2</v>
+      </c>
+      <c r="E22" s="1">
+        <v>-0.29199999999999998</v>
+      </c>
+      <c r="F22" s="1">
+        <v>0.22701099999999999</v>
+      </c>
+      <c r="G22" s="1">
+        <v>271939.46899999998</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="38"/>
+      <c r="B23" s="10">
+        <v>19</v>
+      </c>
+      <c r="C23" s="1">
+        <v>5.7670000000000003</v>
+      </c>
+      <c r="D23" s="1">
+        <v>-1.2E-2</v>
+      </c>
+      <c r="E23" s="1">
+        <v>0.26200000000000001</v>
+      </c>
+      <c r="F23" s="1">
+        <v>0.12518499999999999</v>
+      </c>
+      <c r="G23" s="1">
+        <v>322650.60499999998</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="38"/>
+      <c r="B24" s="10">
+        <v>20</v>
+      </c>
+      <c r="C24" s="1">
+        <v>5.7480000000000002</v>
+      </c>
+      <c r="D24" s="1">
+        <v>-1.9E-2</v>
+      </c>
+      <c r="E24" s="1">
+        <v>-4.3999999999999997E-2</v>
+      </c>
+      <c r="F24" s="1">
+        <v>0.17624899999999999</v>
+      </c>
+      <c r="G24" s="1">
+        <v>408611.29700000002</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="38"/>
+      <c r="B25" s="10">
+        <v>21</v>
+      </c>
+      <c r="C25" s="1">
+        <v>5.7309999999999999</v>
+      </c>
+      <c r="D25" s="1">
+        <v>-1.7000000000000001E-2</v>
+      </c>
+      <c r="E25" s="1">
+        <v>-0.43</v>
+      </c>
+      <c r="F25" s="1">
+        <v>0.25907599999999997</v>
+      </c>
+      <c r="G25" s="1">
+        <v>516119.56300000002</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="38"/>
+      <c r="B26" s="10">
+        <v>22</v>
+      </c>
+      <c r="C26" s="1">
+        <v>5.7140000000000004</v>
+      </c>
+      <c r="D26" s="1">
+        <v>-1.7000000000000001E-2</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="38"/>
+      <c r="B27" s="10">
+        <v>23</v>
+      </c>
+      <c r="C27" s="1">
+        <v>5.7060000000000004</v>
+      </c>
+      <c r="D27" s="1">
+        <v>-8.0000000000000002E-3</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="38"/>
+      <c r="B28" s="10">
+        <v>24</v>
+      </c>
+      <c r="C28" s="1">
+        <v>5.7</v>
+      </c>
+      <c r="D28" s="1">
+        <v>-6.0000000000000001E-3</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="38"/>
+      <c r="B29" s="10">
+        <v>25</v>
+      </c>
+      <c r="C29" s="1">
+        <v>5.6820000000000004</v>
+      </c>
+      <c r="D29" s="1">
+        <v>-1.7999999999999999E-2</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="38"/>
+      <c r="B30" s="10">
+        <v>26</v>
+      </c>
+      <c r="C30" s="1">
+        <v>5.6790000000000003</v>
+      </c>
+      <c r="D30" s="1">
+        <v>-3.0000000000000001E-3</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="38"/>
+      <c r="B31" s="10">
+        <v>27</v>
+      </c>
+      <c r="C31" s="1">
+        <v>5.6680000000000001</v>
+      </c>
+      <c r="D31" s="1">
+        <v>-1.0999999999999999E-2</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="38"/>
+      <c r="B32" s="10">
+        <v>28</v>
+      </c>
+      <c r="C32" s="1">
+        <v>5.6539999999999999</v>
+      </c>
+      <c r="D32" s="1">
+        <v>-1.4E-2</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="38"/>
+      <c r="B33" s="10">
+        <v>29</v>
+      </c>
+      <c r="C33" s="1">
+        <v>5.6529999999999996</v>
+      </c>
+      <c r="D33" s="1">
+        <v>-1E-3</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="38"/>
+      <c r="B34" s="10">
+        <v>30</v>
+      </c>
+      <c r="C34" s="1">
+        <v>5.6449999999999996</v>
+      </c>
+      <c r="D34" s="1">
+        <v>-8.0000000000000002E-3</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="38" t="s">
+        <v>169</v>
+      </c>
+      <c r="B35" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>308</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" s="38"/>
+      <c r="B36" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D36" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>375</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" s="38"/>
+      <c r="B37" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>376</v>
+      </c>
+      <c r="D37" s="7" t="s">
+        <v>311</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="18" x14ac:dyDescent="0.25">
+      <c r="A38" s="38"/>
+      <c r="B38" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D38" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="38"/>
+      <c r="B39" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>378</v>
+      </c>
+      <c r="D39" s="7" t="s">
+        <v>314</v>
+      </c>
+      <c r="E39" s="7"/>
+      <c r="F39" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G39" s="1" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="38"/>
+      <c r="B40" s="10" t="s">
+        <v>297</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D40" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E40" s="7"/>
+      <c r="F40" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G40" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="38"/>
+      <c r="B41" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="D41" s="7" t="s">
+        <v>317</v>
+      </c>
+      <c r="E41" s="7"/>
+      <c r="F41" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G41" s="1" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="38"/>
+      <c r="B42" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D42" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E42" s="7"/>
+      <c r="F42" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G42" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="38"/>
+      <c r="B43" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>381</v>
+      </c>
+      <c r="D43" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="E43" s="7"/>
+      <c r="F43" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G43" s="1" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="38"/>
+      <c r="B44" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>383</v>
+      </c>
+      <c r="D44" s="7" t="s">
+        <v>323</v>
+      </c>
+      <c r="E44" s="7"/>
+      <c r="F44" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G44" s="1" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="38"/>
+      <c r="B45" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>385</v>
+      </c>
+      <c r="D45" s="7" t="s">
+        <v>326</v>
+      </c>
+      <c r="E45" s="7"/>
+      <c r="F45" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G45" s="1" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="38"/>
+      <c r="B46" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="D46" s="7" t="s">
+        <v>329</v>
+      </c>
+      <c r="E46" s="7"/>
+      <c r="F46" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="38"/>
+      <c r="B47" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D47" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E47" s="7"/>
+      <c r="F47" s="1" t="s">
+        <v>389</v>
+      </c>
+      <c r="G47" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="38"/>
+      <c r="B48" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="D48" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="E48" s="7"/>
+      <c r="F48" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G48" s="1" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="38"/>
+      <c r="B49" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>392</v>
+      </c>
+      <c r="D49" s="7" t="s">
+        <v>336</v>
+      </c>
+      <c r="E49" s="7"/>
+      <c r="F49" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G49" s="1" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="38"/>
+      <c r="B50" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="D50" s="7" t="s">
+        <v>339</v>
+      </c>
+      <c r="E50" s="7"/>
+      <c r="F50" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G50" s="1" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="38"/>
+      <c r="B51" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>396</v>
+      </c>
+      <c r="D51" s="7" t="s">
+        <v>342</v>
+      </c>
+      <c r="E51" s="7"/>
+      <c r="F51" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G51" s="1" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="38"/>
+      <c r="B52" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="D52" s="7" t="s">
+        <v>345</v>
+      </c>
+      <c r="E52" s="7"/>
+      <c r="F52" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G52" s="1" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="38"/>
+      <c r="B53" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>400</v>
+      </c>
+      <c r="D53" s="7" t="s">
+        <v>348</v>
+      </c>
+      <c r="E53" s="7"/>
+      <c r="F53" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G53" s="1" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="38"/>
+      <c r="B54" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="D54" s="7" t="s">
+        <v>351</v>
+      </c>
+      <c r="E54" s="7"/>
+      <c r="F54" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G54" s="1" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="38"/>
+      <c r="B55" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D55" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E55" s="7"/>
+      <c r="F55" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G55" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="38"/>
+      <c r="B56" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="D56" s="7" t="s">
+        <v>354</v>
+      </c>
+      <c r="E56" s="7"/>
+      <c r="F56" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G56" s="1" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="38"/>
+      <c r="B57" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="D57" s="7" t="s">
+        <v>357</v>
+      </c>
+      <c r="E57" s="7"/>
+      <c r="F57" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G57" s="1" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="38"/>
+      <c r="B58" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="D58" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="E58" s="7"/>
+      <c r="F58" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G58" s="1" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="38"/>
+      <c r="B59" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D59" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E59" s="7"/>
+      <c r="F59" s="1" t="s">
+        <v>406</v>
+      </c>
+      <c r="G59" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A60" s="38"/>
+      <c r="B60" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>407</v>
+      </c>
+      <c r="D60" s="7" t="s">
+        <v>362</v>
+      </c>
+      <c r="F60" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G60" s="1" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A61" s="38"/>
+      <c r="B61" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>409</v>
+      </c>
+      <c r="D61" s="7" t="s">
+        <v>365</v>
+      </c>
+      <c r="F61" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G61" s="1" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A62" s="38"/>
+      <c r="B62" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>411</v>
+      </c>
+      <c r="D62" s="7" t="s">
+        <v>368</v>
+      </c>
+      <c r="F62" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G62" s="1" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A63" s="38"/>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A64" s="38"/>
+      <c r="B64" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="D64" s="7" t="s">
+        <v>371</v>
+      </c>
+      <c r="F64" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G64" s="1" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A65" s="38" t="s">
+        <v>236</v>
+      </c>
+      <c r="B65" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>415</v>
+      </c>
+      <c r="D65" s="29" t="s">
+        <v>308</v>
+      </c>
+      <c r="E65" s="29"/>
+      <c r="G65" s="1" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A66" s="38"/>
+      <c r="B66" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D66" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="E66" s="29"/>
+      <c r="F66" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G66" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A67" s="38"/>
+      <c r="B67" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>417</v>
+      </c>
+      <c r="D67" s="29" t="s">
+        <v>311</v>
+      </c>
+      <c r="E67" s="29"/>
+      <c r="F67" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G67" s="1" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" s="1" customFormat="1" ht="18" x14ac:dyDescent="0.25">
+      <c r="A68" s="38"/>
+      <c r="B68" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D68" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="E68" s="29"/>
+      <c r="F68" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="G68" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A69" s="38"/>
+      <c r="B69" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>418</v>
+      </c>
+      <c r="D69" s="29" t="s">
+        <v>314</v>
+      </c>
+      <c r="E69" s="29"/>
+      <c r="F69" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G69" s="1" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A70" s="38"/>
+      <c r="B70" s="10" t="s">
+        <v>297</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D70" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="E70" s="29"/>
+      <c r="F70" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G70" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A71" s="38"/>
+      <c r="B71" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>419</v>
+      </c>
+      <c r="D71" s="29" t="s">
+        <v>317</v>
+      </c>
+      <c r="E71" s="29"/>
+      <c r="F71" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G71" s="1" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A72" s="38"/>
+      <c r="B72" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D72" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="E72" s="29"/>
+      <c r="F72" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G72" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A73" s="38"/>
+      <c r="B73" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="C73" s="1" t="s">
+        <v>420</v>
+      </c>
+      <c r="D73" s="29" t="s">
+        <v>320</v>
+      </c>
+      <c r="E73" s="29"/>
+      <c r="F73" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G73" s="1" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A74" s="38"/>
+      <c r="B74" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="C74" s="1" t="s">
+        <v>422</v>
+      </c>
+      <c r="D74" s="29" t="s">
+        <v>323</v>
+      </c>
+      <c r="E74" s="29"/>
+      <c r="F74" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G74" s="1" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A75" s="38"/>
+      <c r="B75" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="C75" s="1" t="s">
+        <v>424</v>
+      </c>
+      <c r="D75" s="29" t="s">
+        <v>326</v>
+      </c>
+      <c r="E75" s="29"/>
+      <c r="F75" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G75" s="1" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A76" s="38"/>
+      <c r="B76" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="C76" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="D76" s="29" t="s">
+        <v>329</v>
+      </c>
+      <c r="E76" s="29"/>
+      <c r="F76" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G76" s="1" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A77" s="38"/>
+      <c r="B77" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D77" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="E77" s="29"/>
+      <c r="F77" s="1" t="s">
+        <v>428</v>
+      </c>
+      <c r="G77" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A78" s="38"/>
+      <c r="B78" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="C78" s="1" t="s">
+        <v>429</v>
+      </c>
+      <c r="D78" s="29" t="s">
+        <v>333</v>
+      </c>
+      <c r="E78" s="29"/>
+      <c r="F78" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G78" s="1" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A79" s="38"/>
+      <c r="B79" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="C79" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="D79" s="29" t="s">
+        <v>336</v>
+      </c>
+      <c r="E79" s="29"/>
+      <c r="F79" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G79" s="1" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A80" s="38"/>
+      <c r="B80" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="C80" s="1" t="s">
+        <v>433</v>
+      </c>
+      <c r="D80" s="29" t="s">
+        <v>339</v>
+      </c>
+      <c r="E80" s="29"/>
+      <c r="F80" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G80" s="1" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A81" s="38"/>
+      <c r="B81" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="C81" s="1" t="s">
+        <v>435</v>
+      </c>
+      <c r="D81" s="29" t="s">
+        <v>342</v>
+      </c>
+      <c r="E81" s="29"/>
+      <c r="F81" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G81" s="1" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="82" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A82" s="38"/>
+      <c r="B82" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="C82" s="1" t="s">
+        <v>437</v>
+      </c>
+      <c r="D82" s="29" t="s">
+        <v>345</v>
+      </c>
+      <c r="E82" s="29"/>
+      <c r="F82" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G82" s="1" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A83" s="38"/>
+      <c r="B83" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>439</v>
+      </c>
+      <c r="D83" s="29" t="s">
+        <v>348</v>
+      </c>
+      <c r="E83" s="29"/>
+      <c r="F83" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G83" s="1" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A84" s="38"/>
+      <c r="B84" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="C84" s="1" t="s">
+        <v>441</v>
+      </c>
+      <c r="D84" s="29" t="s">
+        <v>351</v>
+      </c>
+      <c r="E84" s="29"/>
+      <c r="F84" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G84" s="1" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A85" s="38"/>
+      <c r="B85" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="C85" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D85" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="E85" s="29"/>
+      <c r="F85" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G85" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A86" s="38"/>
+      <c r="B86" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="C86" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="D86" s="29" t="s">
+        <v>354</v>
+      </c>
+      <c r="E86" s="29"/>
+      <c r="F86" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G86" s="1" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A87" s="38"/>
+      <c r="B87" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="C87" s="1" t="s">
+        <v>444</v>
+      </c>
+      <c r="D87" s="29" t="s">
+        <v>357</v>
+      </c>
+      <c r="E87" s="29"/>
+      <c r="F87" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G87" s="1" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A88" s="38"/>
+      <c r="B88" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="C88" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="D88" s="29" t="s">
+        <v>359</v>
+      </c>
+      <c r="E88" s="29"/>
+      <c r="F88" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G88" s="1" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A89" s="38"/>
+      <c r="B89" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="C89" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D89" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="E89" s="29"/>
+      <c r="F89" s="1" t="s">
+        <v>446</v>
+      </c>
+      <c r="G89" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A90" s="38"/>
+      <c r="B90" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="C90" s="1" t="s">
+        <v>447</v>
+      </c>
+      <c r="D90" s="29" t="s">
+        <v>362</v>
+      </c>
+      <c r="E90" s="29"/>
+      <c r="F90" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G90" s="1" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A91" s="38"/>
+      <c r="B91" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="C91" s="1" t="s">
+        <v>449</v>
+      </c>
+      <c r="D91" s="29" t="s">
+        <v>365</v>
+      </c>
+      <c r="E91" s="29"/>
+      <c r="F91" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G91" s="1" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A92" s="38"/>
+      <c r="D92" s="29"/>
+      <c r="E92" s="29"/>
+    </row>
+    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A93" s="38"/>
+      <c r="B93" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="C93" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="D93" s="29" t="s">
+        <v>368</v>
+      </c>
+      <c r="E93" s="29"/>
+      <c r="F93" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G93" s="1" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="94" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A94" s="39"/>
+      <c r="B94" s="33" t="s">
+        <v>154</v>
+      </c>
+      <c r="C94" s="31" t="s">
+        <v>453</v>
+      </c>
+      <c r="D94" s="32" t="s">
+        <v>371</v>
+      </c>
+      <c r="E94" s="32"/>
+      <c r="F94" s="31" t="s">
+        <v>35</v>
+      </c>
+      <c r="G94" s="31" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A96" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C96" s="7"/>
+      <c r="D96" s="1"/>
+      <c r="E96" s="1"/>
+      <c r="J96" s="12"/>
+    </row>
+    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A97" s="12" t="s">
+        <v>509</v>
+      </c>
+      <c r="C97" s="7"/>
+      <c r="D97" s="1"/>
+      <c r="E97" s="1"/>
+      <c r="J97" s="12"/>
+    </row>
+    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A98" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="C98" s="7"/>
+      <c r="D98" s="1"/>
+      <c r="E98" s="1"/>
+      <c r="J98" s="12"/>
+    </row>
+    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A99" s="12" t="s">
+        <v>300</v>
+      </c>
+      <c r="C99" s="7"/>
+      <c r="D99" s="1"/>
+      <c r="E99" s="1"/>
+      <c r="J99" s="12"/>
+    </row>
+    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A100" s="12" t="s">
+        <v>507</v>
+      </c>
+      <c r="C100" s="7"/>
+      <c r="D100" s="1"/>
+      <c r="E100" s="1"/>
+      <c r="J100" s="12"/>
+    </row>
+    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A101" s="21" t="s">
+        <v>301</v>
+      </c>
+      <c r="C101" s="7"/>
+      <c r="D101" s="1"/>
+      <c r="E101" s="1"/>
+      <c r="J101" s="12"/>
+    </row>
+    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A102" s="12" t="s">
+        <v>302</v>
+      </c>
+      <c r="C102" s="7"/>
+      <c r="D102" s="1"/>
+      <c r="E102" s="1"/>
+      <c r="J102" s="12"/>
+    </row>
+    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A103" s="12" t="s">
+        <v>303</v>
+      </c>
+      <c r="C103" s="7"/>
+      <c r="D103" s="1"/>
+      <c r="E103" s="1"/>
+      <c r="J103" s="12"/>
+    </row>
+    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A104" s="12" t="s">
+        <v>510</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="A5:A34"/>
+    <mergeCell ref="A35:A64"/>
+    <mergeCell ref="A65:A94"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010064E03803A74B364DAEBC39F6C7EEC88B" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="49ce98d08d805b506bcc40b8f43aa161">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7096755d-09e2-49ab-9780-382f17a74ff2" xmlns:ns3="2496ba1d-a99b-4e00-82bd-3ea232f3a0a7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d262d534f3278ea9c672dc9f1d9c575b" ns2:_="" ns3:_="">
     <xsd:import namespace="7096755d-09e2-49ab-9780-382f17a74ff2"/>
@@ -7251,15 +9178,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9135FDFF-2234-4F0B-B4DA-2AE6D09006AB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4EBA38C6-46F4-4280-94E3-1F9DA4BE2039}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7276,4 +9204,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9135FDFF-2234-4F0B-B4DA-2AE6D09006AB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>